<commit_message>
Scorecard v3 + cấu hình online + scorecard v2 theo nghiên cứu; các tab chỉ xem số
- Scorecard: gauge, kỳ so sánh, tải PDF/Word, AI comment theo từng tab (tác động lên VN)
- Cấu hình scorecard online: CONFIG_PASSWORD + Google Sheets, lịch sử, hoàn tác
- 3 bộ: Theo dõi BĐS (Nhà ở, KCN), Tỷ giá và Lãi suất, Giá năng lượng; biến chọn theo
  nghiên cứu (IMF Article IV, EMP, EIA, BoC) và phản biện; mốc [giả định] chờ QTRR
- Chuỗi mới: chênh lệch lãi VND−USD, Brent quy ra VND; cách đo % lệch so TB N năm
- FedWatch: số lần kỳ vọng tăng/giảm 12 tháng tới
- Các tab khác chỉ xem số liệu, bỏ trang Ngưỡng

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cache/lme.xlsx
+++ b/data/cache/lme.xlsx
@@ -485,7 +485,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-09T06:56:09+00:00</t>
+          <t>2026-10-09T15:29:42+00:00</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -514,7 +514,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-09T06:56:09+00:00</t>
+          <t>2026-10-09T15:29:42+00:00</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -543,7 +543,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-09T06:56:09+00:00</t>
+          <t>2026-10-09T15:29:42+00:00</t>
         </is>
       </c>
       <c r="D4" t="n">

</xml_diff>